<commit_message>
feat(audit): migrate S1-F02 summary metadata fields
</commit_message>
<xml_diff>
--- a/audit-core/tests/fixtures/s1_region_summary_template.xlsx
+++ b/audit-core/tests/fixtures/s1_region_summary_template.xlsx
@@ -8,11 +8,14 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Meta" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="任意行汇总区域">'Data'!$B$4:$C$4</definedName>
     <definedName name="固定行汇总区域">'Data'!$B$4:$C$6</definedName>
     <definedName name="表头区域">'Data'!$B$2:$C$3</definedName>
+    <definedName name="全局单元格区域.批次">'Meta'!$A$1</definedName>
+    <definedName name="单元格区域.分组" localSheetId="0">'Data'!$F$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -417,9 +420,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:C7"/>
+  <dimension ref="B1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="1">
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>local metadata cell</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
       <c r="B2" t="inlineStr">
         <is>
@@ -485,4 +495,25 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>global metadata cell</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>